<commit_message>
Correction bugs disciplineEquipementSocial, Practitioner.qualification:exercicePro (#186)
* update disciplineequipementsocial

* update exercicePro 742d61209b8528288c62bd919fbb7c8e1a149f0f
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-dp-healthcareservice-social-equipment.xlsx
+++ b/main/ig/StructureDefinition-as-dp-healthcareservice-social-equipment.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-19T13:42:29+00:00</t>
+    <t>2024-03-04T16:55:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -780,7 +780,7 @@
 </t>
   </si>
   <si>
-    <t>La discipline déterminant la nature de l’activité (disciplineEquipementSociale).</t>
+    <t>Broad category of service being performed or delivered</t>
   </si>
   <si>
     <t>Identifies the broad category of service being performed or delivered.</t>
@@ -808,7 +808,7 @@
 </t>
   </si>
   <si>
-    <t>Type of service that may be delivered or performed</t>
+    <t>La discipline déterminant la nature de l’activité (disciplineEquipementSociale).</t>
   </si>
   <si>
     <t>The specific type of service that may be delivered or performed.</t>
@@ -4462,7 +4462,7 @@
         <v>76</v>
       </c>
       <c r="H27" t="s" s="2">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="I27" t="s" s="2">
         <v>75</v>
@@ -4570,7 +4570,7 @@
         <v>77</v>
       </c>
       <c r="H28" t="s" s="2">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="I28" t="s" s="2">
         <v>75</v>

</xml_diff>